<commit_message>
add facilities, environment, and rcr
</commit_message>
<xml_diff>
--- a/checklist.xlsx
+++ b/checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timbarry/research_code/crispr_safe_parent/k99_revision/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C75A0C92-0245-DA4B-BAC7-046804705903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40C14992-83AD-B946-B28E-6DCE13DDE05B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" xr2:uid="{F7FD2756-E949-F24E-A11D-D83B080FEEE6}"/>
   </bookViews>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
-  <si>
-    <t>Cover Letter</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>Project Summary/Abstract</t>
   </si>
@@ -530,14 +527,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17E6DA6-B7A7-E844-9411-6C95D185F317}">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="34" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="163.6640625" style="3" customWidth="1"/>
     <col min="2" max="2" width="69.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="31" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -548,7 +545,7 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
     </row>
-    <row r="2" spans="1:7" ht="31" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -559,7 +556,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -570,18 +567,20 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="37" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -592,7 +591,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:7" ht="37" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -603,7 +602,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
     </row>
-    <row r="7" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -614,8 +613,8 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
     </row>
-    <row r="8" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="3"/>
@@ -625,8 +624,8 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
     </row>
-    <row r="9" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="3"/>
@@ -636,7 +635,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -647,7 +646,7 @@
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
     </row>
-    <row r="11" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -669,8 +668,8 @@
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="3"/>
@@ -680,8 +679,8 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
     </row>
-    <row r="14" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:7" ht="41" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B14" s="3"/>
@@ -691,18 +690,20 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
     </row>
-    <row r="15" spans="1:7" ht="41" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="3"/>
+      <c r="B15" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
@@ -713,10 +714,8 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
     </row>
-    <row r="17" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="1" t="s">
-        <v>16</v>
-      </c>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A17" s="1"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -725,8 +724,12 @@
       <c r="G17" s="3"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A18" s="1"/>
-      <c r="B18" s="3"/>
+      <c r="A18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
@@ -735,24 +738,17 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="B20" s="3"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
@@ -761,29 +757,29 @@
       <c r="B21" s="3"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A22" s="3" t="s">
+      <c r="B22" s="3"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="3"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="B23" s="3"/>
+      <c r="B23" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="B25" s="3"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
@@ -792,24 +788,24 @@
       <c r="B26" s="3"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A27" s="3" t="s">
+      <c r="B27" s="3"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A28" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="3"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B28" s="3"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A29" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="3"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A30" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="B30" s="3"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A31" s="3" t="s">
@@ -818,27 +814,21 @@
       <c r="B31" s="3"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A32" s="3" t="s">
+      <c r="B32" s="3"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A33" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="3"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B33" s="3"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A34" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A35" s="3" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A36" s="3" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update research sharing and phs form
</commit_message>
<xml_diff>
--- a/checklist.xlsx
+++ b/checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timbarry/research_code/crispr_safe_parent/k99_revision/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40C14992-83AD-B946-B28E-6DCE13DDE05B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B90AECAE-34B0-1C47-839E-448F59B4EF8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" xr2:uid="{F7FD2756-E949-F24E-A11D-D83B080FEEE6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>Project Summary/Abstract</t>
   </si>
@@ -53,9 +53,6 @@
     <t>Facilities &amp; Other Resources</t>
   </si>
   <si>
-    <t>Other Attachments</t>
-  </si>
-  <si>
     <t>Biosketch</t>
   </si>
   <si>
@@ -138,13 +135,19 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Document</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -155,23 +158,43 @@
     <font>
       <sz val="26"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="26"/>
+      <sz val="24"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -186,13 +209,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,305 +558,316 @@
   <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="34" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="163.6640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="163.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="69.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="31" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="32" x14ac:dyDescent="0.4">
+      <c r="A1" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="31" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-    </row>
-    <row r="5" spans="1:7" ht="37" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="4"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-    </row>
-    <row r="7" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="s">
+      <c r="B7" s="4"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-    </row>
-    <row r="8" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-    </row>
-    <row r="10" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A11" s="1" t="s">
+      <c r="B11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-    </row>
-    <row r="13" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" ht="41" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-    </row>
-    <row r="14" spans="1:7" ht="41" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A15" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A15" s="1" t="s">
+      <c r="B15" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-    </row>
-    <row r="16" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A17" s="5"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A17" s="1"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A18" s="3" t="s">
+      <c r="B18" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+    </row>
+    <row r="19" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A19" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A19" s="3" t="s">
+      <c r="B19" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A20" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A20" s="3" t="s">
+      <c r="B20" s="7"/>
+    </row>
+    <row r="21" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A21" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="3"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A21" s="3" t="s">
+      <c r="B21" s="7"/>
+    </row>
+    <row r="22" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+    </row>
+    <row r="23" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A23" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="3"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="B22" s="3"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A23" s="3" t="s">
+      <c r="B23" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A24" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A24" s="3" t="s">
+      <c r="B24" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A25" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A25" s="3" t="s">
+      <c r="B25" s="7"/>
+    </row>
+    <row r="26" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A26" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="3"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A26" s="3" t="s">
+      <c r="B26" s="7"/>
+    </row>
+    <row r="27" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
+    </row>
+    <row r="28" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A28" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="3"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="B27" s="3"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A28" s="3" t="s">
+      <c r="B28" s="7"/>
+    </row>
+    <row r="29" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A29" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="3"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A29" s="3" t="s">
+      <c r="B29" s="7"/>
+    </row>
+    <row r="30" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A30" s="7" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A30" s="3" t="s">
+      <c r="B30" s="7"/>
+    </row>
+    <row r="31" spans="1:7" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="A31" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B30" s="3"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A31" s="3" t="s">
+      <c r="B31" s="7"/>
+    </row>
+    <row r="32" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="3"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="B32" s="3"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A33" s="3" t="s">
+    </row>
+    <row r="34" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A34" s="3" t="s">
+    <row r="35" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="2" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A35" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>